<commit_message>
reworked the logic and amended the structure of the script
</commit_message>
<xml_diff>
--- a/DataFile/datafile.xlsx
+++ b/DataFile/datafile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x1016008\PycharmProjects\ShopB2Wise\DataFile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D03519-6CAB-4A30-A657-11F08A027279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE2A2A9-408B-4570-AB0C-1A2DAD38B256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Addition" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="40">
   <si>
     <t>TestCase</t>
   </si>
@@ -477,12 +477,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
@@ -494,11 +494,11 @@
     <col min="13" max="13" width="9" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="5" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -551,7 +551,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -604,7 +604,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>29</v>
       </c>
@@ -612,13 +612,13 @@
         <v>18</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3" t="s">
         <v>31</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
@@ -654,10 +654,10 @@
         <v>32</v>
       </c>
       <c r="Q3">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>30</v>
       </c>
@@ -665,7 +665,7 @@
         <v>18</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" t="s">
         <v>31</v>
@@ -677,37 +677,37 @@
         <v>33</v>
       </c>
       <c r="G4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H4" t="s">
         <v>34</v>
       </c>
       <c r="I4">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J4" t="s">
         <v>35</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L4" t="s">
         <v>36</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N4" t="s">
         <v>27</v>
       </c>
       <c r="O4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P4" t="s">
         <v>32</v>
       </c>
       <c r="Q4">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -720,36 +720,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B666F93E-0D52-4998-B04F-BF60BB25635F}">
   <dimension ref="A1:Y4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="68.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="68.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="5" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="5" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="5" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -826,9 +826,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
@@ -840,10 +840,10 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2">
-        <v>6</v>
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -903,9 +903,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
@@ -914,7 +914,7 @@
         <v>6</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E3" t="s">
         <v>27</v>
@@ -923,7 +923,7 @@
         <v>6</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H3" t="s">
         <v>17</v>
@@ -980,9 +980,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>
@@ -991,7 +991,7 @@
         <v>6</v>
       </c>
       <c r="D4">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E4" t="s">
         <v>27</v>
@@ -1000,7 +1000,7 @@
         <v>6</v>
       </c>
       <c r="G4">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H4" t="s">
         <v>17</v>

</xml_diff>